<commit_message>
colors token and sequence
</commit_message>
<xml_diff>
--- a/results/manual_eval_qwen14B_rag_sequence_validation.xlsx
+++ b/results/manual_eval_qwen14B_rag_sequence_validation.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\YADEL\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\RAG\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13528CB6-EBFB-40DB-A640-2EBFCEB3B516}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE057D8F-C078-4F77-A232-B3D1E702B4CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2842,6 +2842,8 @@
   <cols>
     <col min="1" max="1" width="17.5546875" customWidth="1"/>
     <col min="2" max="2" width="20.33203125" customWidth="1"/>
+    <col min="6" max="6" width="22.6640625" customWidth="1"/>
+    <col min="7" max="7" width="35.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">

</xml_diff>